<commit_message>
Read Remita payroll purpose, simplify sheet suggested reason (Salary, Allowances, Gift (birthday), Check: ...)
</commit_message>
<xml_diff>
--- a/review/Adepeju-Popoola-income-review.xlsx
+++ b/review/Adepeju-Popoola-income-review.xlsx
@@ -430,10 +430,10 @@
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -510,16 +510,19 @@
       <c r="D3" t="n">
         <v>654072</v>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Staff salary for March 2026</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
           <t>REMITA INFLOW R-1445788162/NIGERIAN U:STAFFSALARYFORMARCH2026:CBN:14457955/90144578 81620</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Business or trade payment</t>
+          <t>Salary, Allowances, Burial assistance, Bonus, 2026 one off productivity recognition</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -529,8 +532,6 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
           <t>Tue Mar 31 2026</t>
@@ -539,19 +540,18 @@
       <c r="D4" t="n">
         <v>3786435</v>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2nd quarter allowances 2026 to staff</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
           <t>REMITA INFLOW R-1450507303/NIGERIAN U:2NDQUARTERALLOWANCES2026TOSTAFF:CBN:/901450 5073030</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>Thu Apr 23 2026</t>
@@ -560,19 +560,18 @@
       <c r="D5" t="n">
         <v>654072</v>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Staff salary for April 2026</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
           <t>REMITA INFLOW R-1458479293/NIGERIAN U:STAFFSALARYFORAPRIL2026:CBN:14586777/9014584792 930</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>Tue May 05 2026</t>
@@ -581,19 +580,18 @@
       <c r="D6" t="n">
         <v>9500000</v>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Annual intervention allowance to NUPRC</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
           <t>REMITA INFLOW R-1463090335/NIGERIAN U:ANNUALINTERVENTIONALLOWANCETONUPRCST/901 4630903350</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>Thu May 07 2026</t>
@@ -602,19 +600,18 @@
       <c r="D7" t="n">
         <v>1077976</v>
       </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Employee family burial assistance</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>REMITA INFLOW R-1464021004/NIGERIAN U:EMPLOYEEFAMILYBURIALASSISTANCE:CBN:1/9014640 210040</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>Fri Jun 26 2026</t>
@@ -623,19 +620,18 @@
       <c r="D8" t="n">
         <v>3786435</v>
       </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>3rd qtr 2026 allowances for NUPRC staff</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
           <t>REMITA INFLOW R-1479557315/NIGERIAN U:3RDQTR2026ALLOWANCESFORNUPRCSTAFF:CB/90147 95573150</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>Sat Aug 29 2026</t>
@@ -644,19 +640,18 @@
       <c r="D9" t="n">
         <v>2155953</v>
       </c>
-      <c r="E9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>End of negotiation bonus 2026</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
           <t>REMITA INFLOW R-1506814400/NIGERIAN U:ENDOFNEGOTIATIONBONUS2026:CBN:150685/90150681 44000</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
           <t>Tue Sep 08 2026</t>
@@ -665,21 +660,18 @@
       <c r="D10" t="n">
         <v>10500000</v>
       </c>
-      <c r="E10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2026 one off productivity recognition</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr">
         <is>
           <t>REMITA INFLOW R-1510509599/NIGERIAN U:2026ONEOFFPRODUCTIVITYRECOGNITIONALL/9015105 095990</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>Subtotal for Nigerian:</t>
@@ -688,10 +680,8 @@
       <c r="F11" t="n">
         <v>32114942.6</v>
       </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
@@ -711,13 +701,11 @@
       <c r="D13" t="n">
         <v>5000000</v>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>ACCOUNT TRANSFERS MOB: TRF FROM AMUSE GAMES AND ENTERTAINMENT 54******0936 TO POPOOLA ADEPEJU ADETUTU - 65******2249 REQUEST</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>Business or trade payment</t>
@@ -730,8 +718,6 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
           <t>Wed Sep 02 2026</t>
@@ -740,21 +726,13 @@
       <c r="D14" t="n">
         <v>500000</v>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>TRANSFER BETWEEN CUSTOMERS TRZL-TRANSFER TO ( POPOOLA ADEPEJU ADETUTU ) FROM ( AMUSE GAMES AND ENTERTAINMENT)|TRF</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>Subtotal for Amuse Games And Entertainment:</t>
@@ -763,10 +741,8 @@
       <c r="F15" t="n">
         <v>5500000</v>
       </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
@@ -786,14 +762,21 @@
       <c r="D17" t="n">
         <v>648358</v>
       </c>
-      <c r="E17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>May 2026 NUPRC staff salary</t>
+        </is>
+      </c>
       <c r="F17" t="inlineStr">
         <is>
           <t>REMITA INFLOW R-1468069461/NIGERIAN U:MAY2026NUPRCSTAFFSALARY:CBN:14681127/90146806 94610</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Salary</t>
+        </is>
+      </c>
       <c r="I17" t="inlineStr">
         <is>
           <t>Needs your review</t>
@@ -801,8 +784,6 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
-      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
           <t>Wed Jun 24 2026</t>
@@ -811,19 +792,18 @@
       <c r="D18" t="n">
         <v>648358</v>
       </c>
-      <c r="E18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Staff salary for June 2026</t>
+        </is>
+      </c>
       <c r="F18" t="inlineStr">
         <is>
           <t>REMITA INFLOW R-1477854687/NIGERIAN U:STAFFSALARYFORJUNE2026:CBN:147836786/9014778546</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr"/>
-      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
           <t>Wed Jul 22 2026</t>
@@ -832,19 +812,18 @@
       <c r="D19" t="n">
         <v>648358</v>
       </c>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Staff salary July 2026</t>
+        </is>
+      </c>
       <c r="F19" t="inlineStr">
         <is>
           <t>REMITA INFLOW R-1490274894/NIGERIAN U:STAFFSALARYJULY2026:CBN:1490899371-:/90149027489 40</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr"/>
-      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
           <t>Mon Aug 24 2026</t>
@@ -853,21 +832,18 @@
       <c r="D20" t="n">
         <v>648358</v>
       </c>
-      <c r="E20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Staff salary for August 2026</t>
+        </is>
+      </c>
       <c r="F20" t="inlineStr">
         <is>
           <t>REMITA INFLOW R-1503656521/NIGERIAN U:STAFFSALARYFORAUGUST2026:CBN:1503593/90150365 65210</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr"/>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
           <t>Subtotal for Salary:</t>
@@ -876,10 +852,8 @@
       <c r="F21" t="n">
         <v>2593433.6</v>
       </c>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
@@ -899,13 +873,11 @@
       <c r="D23" t="n">
         <v>2000000</v>
       </c>
-      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>INWARD TRANSFER (N) FROM WEMA/ DENTIST AT YOUR DOOR DENTAL CLINIC_6507032249-EVENT FUNDS/000017260511130927856109490448</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>Business or trade payment</t>
@@ -918,8 +890,6 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr"/>
-      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
           <t>Tue May 26 2026</t>
@@ -928,21 +898,13 @@
       <c r="D24" t="n">
         <v>500000</v>
       </c>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>INWARD TRANSFER (N) FROM WEMA/ DENTIST AT YOUR DOOR DENTAL CLINIC_6507032249-BO DENTIST AT YOUR D IFO POPOOLA ADEPEJU ADETUTU/000017260526150812965632837705</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr"/>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
           <t>Subtotal for Dentist At Your Door Dental Clinic:</t>
@@ -951,10 +913,8 @@
       <c r="F25" t="n">
         <v>2500000</v>
       </c>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
@@ -974,19 +934,13 @@
       <c r="D27" t="n">
         <v>200000</v>
       </c>
-      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>INWARD TRANSFER (N) FROM STERLING/ ADEPEJU ADETUTU POPOOLA-ONEBANK TRANSFER FROM ADEPEJU ADETUTU POPOOLA TO POPOOLA ADEPEJU ADET/000001260717150805522583125499</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr"/>
-      <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
           <t>Wed Jul 22 2026</t>
@@ -995,19 +949,13 @@
       <c r="D28" t="n">
         <v>1000000</v>
       </c>
-      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>INWARD TRANSFER (N) FROM FBN/ POPOOLA ADEPEJU ADETUTU-FIPIBPSPOPOOLA ADEPEJU ADPHUBOUTWARD23015711POPOOLA ADEPEJU ADETUTUPOPOPOP/000016260722142819002399411432</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr"/>
-      <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
           <t>Tue Aug 11 2026</t>
@@ -1016,21 +964,13 @@
       <c r="D29" t="n">
         <v>800000</v>
       </c>
-      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>INWARD TRANSFER (N) FROM FBN/ POPOOLA ADEPEJU ADETUTU-FIPBRPOPOOLA ADEPEJU ADTRFPOPOOLA ADEPEJU AD/000016260811133458002522214027</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr"/>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
           <t>Subtotal for Self (transfers from your own name/account):</t>
@@ -1039,10 +979,8 @@
       <c r="F30" t="n">
         <v>2000000</v>
       </c>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
@@ -1062,14 +1000,11 @@
       <c r="D32" t="n">
         <v>250000</v>
       </c>
-      <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
           <t>INWARD TRANSFER(H) FROM OPAY/ OLUWAYEMISI WASILAT AKINTONWA-TRANSFER FROM OLUWAYEMISI W/100004260405211613156502708324</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
           <t>Needs your review</t>
@@ -1077,8 +1012,6 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr"/>
-      <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
           <t>Tue Jun 16 2026</t>
@@ -1087,19 +1020,13 @@
       <c r="D33" t="n">
         <v>100000</v>
       </c>
-      <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
           <t>INWARD TRANSFER (N) FROM STERLING/ OLUWAYEMISI WASILAT AKINTONWA-ONEBANK TRANSFER FROM OLUWAYEMISI WASILAT AKINTONWA TO POPOOLA /000001260616180926530627186667</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr"/>
-      <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
           <t>Tue Jun 23 2026</t>
@@ -1108,19 +1035,13 @@
       <c r="D34" t="n">
         <v>300000</v>
       </c>
-      <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
           <t>INWARD TRANSFER (N) FROM STERLING/ OLUWAYEMISI WASILAT AKINTONWA-ONEBANKTRANSFERFROMOLUWAYEMISI WASILATAKINTONWATOPOPOOLAADEPEJUA/000001260 623134216310682777889</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr"/>
-      <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
           <t>Fri Jun 26 2026</t>
@@ -1129,19 +1050,13 @@
       <c r="D35" t="n">
         <v>300000</v>
       </c>
-      <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
           <t>INWARD TRANSFER (N) FROM STERLING/ OLUWAYEMISI WASILAT AKINTONWA-ONEBANKTRANSFERFROMOLUWAYEMISI WASILATAKINTONWATOPOPOOLAADEPEJUA/000001260 626145431272563810095</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr"/>
-      <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
           <t>Sat Aug 08 2026</t>
@@ -1150,19 +1065,13 @@
       <c r="D36" t="n">
         <v>500000</v>
       </c>
-      <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
           <t>INWARD TRANSFER (N) FROM STERLING/ OLUWAYEMISI WASILAT AKINTONWA-ONEBANK TRANSFER FROM OLUWAYEMISI WASILAT AKINTONWA TO POPOOLA /000001260808134809150694488967</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr"/>
-      <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
           <t>Sat Aug 08 2026</t>
@@ -1171,19 +1080,13 @@
       <c r="D37" t="n">
         <v>300000</v>
       </c>
-      <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
           <t>INWARD TRANSFER (N) FROM STERLING/ OLUWAYEMISI WASILAT AKINTONWA-ONEBANK TRANSFER FROM OLUWAYEMISI WASILAT AKINTONWA TO POPOOLA /000001260808135213116475951589</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr"/>
-      <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
           <t>Sat Aug 08 2026</t>
@@ -1192,21 +1095,13 @@
       <c r="D38" t="n">
         <v>200000</v>
       </c>
-      <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr">
         <is>
           <t>INWARD TRANSFER (N) FROM STERLING/ OLUWAYEMISI WASILAT AKINTONWA-ONEBANK TRANSFER FROM OLUWAYEMISI WASILAT AKINTONWA TO POPOOLA /000001260808135256375156196088</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr"/>
-      <c r="B39" t="inlineStr"/>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
           <t>Subtotal for Oluwayemisi Wasilat Akintonwa:</t>
@@ -1215,10 +1110,8 @@
       <c r="F39" t="n">
         <v>1950000</v>
       </c>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="40"/>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
@@ -1238,14 +1131,11 @@
       <c r="D41" t="n">
         <v>150000</v>
       </c>
-      <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
         <is>
           <t>INWARD TRANSFER (N) FROM STERLING/ DAVID AND ADENIKE POPOOLA-ONEBANK TRANSFER FROM DAVID AND ADENIKE POPOOLA TO POPOOLA ADEPEJU /000001260619205827710535536297</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr">
         <is>
           <t>Needs your review</t>
@@ -1253,10 +1143,6 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr"/>
-      <c r="B42" t="inlineStr"/>
-      <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
           <t>Subtotal for David And Adenike Popoola:</t>
@@ -1265,10 +1151,8 @@
       <c r="F42" t="n">
         <v>150000</v>
       </c>
-      <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="43"/>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
@@ -1288,16 +1172,14 @@
       <c r="D44" t="n">
         <v>50000</v>
       </c>
-      <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
         <is>
           <t>INWARD TRANSFER(H) FROM GTBANK/ LADENIKA ADEBOWALE-HAPPY BIRTHDAY SIS TO POPOOLA ADEPE/000013260513230416000026801405</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Gift</t>
+          <t>Gift (birthday)</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -1307,10 +1189,6 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr"/>
-      <c r="B45" t="inlineStr"/>
-      <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
           <t>Subtotal for Ladenika Adebowale:</t>
@@ -1319,15 +1197,9 @@
       <c r="F45" t="n">
         <v>50000</v>
       </c>
-      <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="46"/>
     <row r="47">
-      <c r="A47" t="inlineStr"/>
-      <c r="B47" t="inlineStr"/>
-      <c r="C47" t="inlineStr"/>
-      <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
           <t>GRAND TOTAL:</t>
@@ -1336,9 +1208,6 @@
       <c r="F47" t="n">
         <v>44858376.2</v>
       </c>
-      <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>